<commit_message>
docs(bhe): observe before formalizing week 5 pedagogical signals
</commit_message>
<xml_diff>
--- a/docs/Word/brick_1.xlsx
+++ b/docs/Word/brick_1.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\david\Documents\Codex\2026-05-03\coucou-mon-gpt-3-c-est\Boost Hyper Engine\docs\Word\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FEF4493-6F0F-4CB8-945B-7B46BCE02D19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92FF0982-65C4-4C90-A45C-C2BAB0C8A9A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="57480" yWindow="15990" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{D149BA85-6973-494D-8FB0-893C49EAA7D2}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="119">
   <si>
     <t>on commence concret/perceptif (images)</t>
   </si>
@@ -421,12 +421,163 @@
   <si>
     <t>Réinvestissement personnel d’une règle</t>
   </si>
+  <si>
+    <t>Transformation de posture ?</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Introduction </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>(learning objectives + roadmap + timing)</t>
+    </r>
+  </si>
+  <si>
+    <t>Orientation / expectation framing / goal projection</t>
+  </si>
+  <si>
+    <t>✅ Oui</t>
+  </si>
+  <si>
+    <t>OrientationMoment (?)</t>
+  </si>
+  <si>
+    <t>Réduction de l’incertitude, annonce du parcours, sens donné aux activités. Pas contenu passif. Prépare cognitivement l’apprentissage.</t>
+  </si>
+  <si>
+    <r>
+      <t>I start</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> — “How do you memorize vocabulary?”</t>
+    </r>
+  </si>
+  <si>
+    <t>Métacognition / self-awareness / learning strategy reflection</t>
+  </si>
+  <si>
+    <t>✅ Très forte</t>
+  </si>
+  <si>
+    <t>ReflectionMoment (?)</t>
+  </si>
+  <si>
+    <t>L’apprenant réfléchit à ses propres stratégies avant l’activité. Très Degache-compatible. Cognition guidée sans évaluation forte immédiate.</t>
+  </si>
+  <si>
+    <r>
+      <t>I learn</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> — découverte d’une stratégie de mémorisation</t>
+    </r>
+  </si>
+  <si>
+    <t>Strategy awareness / guided conceptualization</t>
+  </si>
+  <si>
+    <t>L’étudiant apprend une méthode d’apprentissage, pas encore le contenu lui-même</t>
+  </si>
+  <si>
+    <r>
+      <t>I practise</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> — construire son spiderweb</t>
+    </r>
+  </si>
+  <si>
+    <t>Construction / personalization / active organization</t>
+  </si>
+  <si>
+    <t>✅ Forte</t>
+  </si>
+  <si>
+    <t>TransformationSet (+)</t>
+  </si>
+  <si>
+    <t>Plusieurs opérations se croisent dans un même moment. Très bon signal de composition cognitive</t>
+  </si>
+  <si>
+    <r>
+      <t>I say</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> — expliquer / partager sa stratégie</t>
+    </r>
+  </si>
+  <si>
+    <t>Verbalisation / explicitation / organization</t>
+  </si>
+  <si>
+    <t>Emerging signal (?)</t>
+  </si>
+  <si>
+    <t>Rendre visible sa compréhension. Très learning-by-teaching compatible</t>
+  </si>
+  <si>
+    <r>
+      <t>Autonomy</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> — réutiliser la méthode</t>
+    </r>
+  </si>
+  <si>
+    <t>Transfer / reuse / autonomy / ownership</t>
+  </si>
+  <si>
+    <t>L’apprentissage sort de la brique et devient réutilisable</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -446,6 +597,14 @@
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial Unicode MS"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -468,7 +627,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -489,6 +648,9 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -870,7 +1032,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="58">
+    <row r="3" spans="1:6" ht="43.5">
       <c r="B3" s="1" t="s">
         <v>3</v>
       </c>
@@ -1028,13 +1190,16 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C62B3E51-9EEE-4F18-8DA7-06BECF96FF04}">
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:G28"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
   <cols>
+    <col min="1" max="1" width="3" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="33.453125" customWidth="1"/>
     <col min="3" max="3" width="32.6328125" customWidth="1"/>
     <col min="4" max="4" width="26.453125" customWidth="1"/>
     <col min="6" max="6" width="32.90625" customWidth="1"/>
+    <col min="7" max="7" width="38.7265625" customWidth="1"/>
+    <col min="8" max="8" width="19.81640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -1297,6 +1462,213 @@
         <v>92</v>
       </c>
     </row>
+    <row r="18" spans="1:7">
+      <c r="A18" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="D18" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="E18" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="F18" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="G18" s="5" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="58">
+      <c r="A19" s="6">
+        <v>1</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="D19" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="E19" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="F19" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="G19" s="6" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="80.5" customHeight="1">
+      <c r="A20" s="6">
+        <v>2</v>
+      </c>
+      <c r="B20" s="8" t="s">
+        <v>99</v>
+      </c>
+      <c r="C20" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="D20" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="E20" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="F20" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="G20" s="6" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7">
+      <c r="A22" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="B22" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="C22" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="D22" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="E22" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="F22" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="G22" s="5" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" ht="43.5">
+      <c r="A23" s="6">
+        <v>3</v>
+      </c>
+      <c r="B23" s="8" t="s">
+        <v>104</v>
+      </c>
+      <c r="C23" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="D23" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="E23" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="F23" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="G23" s="6" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" ht="43.5">
+      <c r="A24" s="6">
+        <v>4</v>
+      </c>
+      <c r="B24" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="C24" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="D24" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="E24" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="F24" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="G24" s="6" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7">
+      <c r="A26" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="B26" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="C26" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="D26" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="E26" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="F26" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="G26" s="5" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" ht="29">
+      <c r="A27" s="6">
+        <v>5</v>
+      </c>
+      <c r="B27" s="8" t="s">
+        <v>112</v>
+      </c>
+      <c r="C27" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="D27" s="7" t="s">
+        <v>114</v>
+      </c>
+      <c r="E27" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="F27" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="G27" s="6" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" ht="29">
+      <c r="A28" s="6">
+        <v>6</v>
+      </c>
+      <c r="B28" s="8" t="s">
+        <v>116</v>
+      </c>
+      <c r="C28" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="D28" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="E28" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="F28" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="G28" s="6" t="s">
+        <v>101</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(authoring): bridge pedagogical uses and BHE representations
</commit_message>
<xml_diff>
--- a/docs/Word/brick_1.xlsx
+++ b/docs/Word/brick_1.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\david\Documents\Codex\2026-05-03\coucou-mon-gpt-3-c-est\Boost Hyper Engine\docs\Word\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92FF0982-65C4-4C90-A45C-C2BAB0C8A9A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E96AF76-501A-4DAB-8853-6EBC60C0116B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="15990" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{D149BA85-6973-494D-8FB0-893C49EAA7D2}"/>
+    <workbookView xWindow="57480" yWindow="15990" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{D149BA85-6973-494D-8FB0-893C49EAA7D2}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
     <sheet name="Feuil2" sheetId="2" r:id="rId2"/>
+    <sheet name="Feuil3" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="149">
   <si>
     <t>on commence concret/perceptif (images)</t>
   </si>
@@ -571,6 +572,96 @@
   </si>
   <si>
     <t>L’apprentissage sort de la brique et devient réutilisable</t>
+  </si>
+  <si>
+    <t>Primitives cognitives</t>
+  </si>
+  <si>
+    <t>PedagogicalObject</t>
+  </si>
+  <si>
+    <t>├── Constructive / Active</t>
+  </si>
+  <si>
+    <t>│   ├── AssociationSet</t>
+  </si>
+  <si>
+    <t>│   ├── ClassificationSet</t>
+  </si>
+  <si>
+    <t>│   ├── SequenceSet</t>
+  </si>
+  <si>
+    <t>│   ├── TransformationSet</t>
+  </si>
+  <si>
+    <t>│   ├── IdentificationSet</t>
+  </si>
+  <si>
+    <t>│   ├── InferenceSet</t>
+  </si>
+  <si>
+    <t>│</t>
+  </si>
+  <si>
+    <t>└── Expositive / Guided</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    ├── DiscoverySequence</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    ├── GuidedObservation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    ├── Contextualization</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    ├── MediaSequence</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    └── ReflectivePrompt</t>
+  </si>
+  <si>
+    <t>- associer</t>
+  </si>
+  <si>
+    <t>- classer</t>
+  </si>
+  <si>
+    <t>- ordonner</t>
+  </si>
+  <si>
+    <t>- identifier</t>
+  </si>
+  <si>
+    <t>- inférer</t>
+  </si>
+  <si>
+    <t>- transformer</t>
+  </si>
+  <si>
+    <t>- mémoriser</t>
+  </si>
+  <si>
+    <t>notice</t>
+  </si>
+  <si>
+    <t>reflect</t>
+  </si>
+  <si>
+    <t>produce</t>
+  </si>
+  <si>
+    <t>compare</t>
+  </si>
+  <si>
+    <t>imitate</t>
+  </si>
+  <si>
+    <t>self-adjust</t>
+  </si>
+  <si>
+    <t>transfer</t>
   </si>
 </sst>
 </file>
@@ -627,7 +718,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -653,6 +744,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1672,4 +1764,159 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3D3AAA32-A13F-4CCB-A864-EBDDD2812E5F}">
+  <dimension ref="C4:G28"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <cols>
+    <col min="3" max="3" width="23.7265625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="4" spans="3:7">
+      <c r="C4" s="9" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="5" spans="3:7">
+      <c r="C5" s="9"/>
+    </row>
+    <row r="6" spans="3:7">
+      <c r="C6" s="9" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="7" spans="3:7">
+      <c r="C7" s="9" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="8" spans="3:7">
+      <c r="C8" s="9" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="9" spans="3:7">
+      <c r="C9" s="9" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="10" spans="3:7">
+      <c r="C10" s="9" t="s">
+        <v>139</v>
+      </c>
+      <c r="G10" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="11" spans="3:7">
+      <c r="C11" s="9" t="s">
+        <v>140</v>
+      </c>
+      <c r="G11" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="12" spans="3:7">
+      <c r="C12" s="9" t="s">
+        <v>141</v>
+      </c>
+      <c r="G12" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="13" spans="3:7">
+      <c r="C13" s="9"/>
+      <c r="G13" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="14" spans="3:7">
+      <c r="C14" s="9" t="s">
+        <v>120</v>
+      </c>
+      <c r="G14" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="15" spans="3:7">
+      <c r="C15" s="9" t="s">
+        <v>121</v>
+      </c>
+      <c r="G15" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="16" spans="3:7">
+      <c r="C16" s="9" t="s">
+        <v>122</v>
+      </c>
+      <c r="G16" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="17" spans="3:3">
+      <c r="C17" s="9" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="18" spans="3:3">
+      <c r="C18" s="9" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="19" spans="3:3">
+      <c r="C19" s="9" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="20" spans="3:3">
+      <c r="C20" s="9" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="21" spans="3:3">
+      <c r="C21" s="9" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="22" spans="3:3">
+      <c r="C22" s="9" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="23" spans="3:3">
+      <c r="C23" s="9" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="24" spans="3:3">
+      <c r="C24" s="9" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="25" spans="3:3">
+      <c r="C25" s="9" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="26" spans="3:3">
+      <c r="C26" s="9" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="27" spans="3:3">
+      <c r="C27" s="9" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="28" spans="3:3">
+      <c r="C28" s="9" t="s">
+        <v>134</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>